<commit_message>
Harden update.sh: scrub xlsx metadata before regenerating
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: add Score column to xlsx, extend live window to 130min, remove sync script
- Add Score col (G) to xlsx as text-formatted manual input
- generate_ics.py reads col G and writes through to scores.json
- live_score_updater.py live window extended from 100 to 130 min (covers ET + penalties)
- Delete sync_scores_to_xlsx.py — scores now flow xlsx → scores.json only
- Add backfill_scores.py for fetching historical ESPN results
- Fix xlsx col G number format to text to prevent score values being parsed as time

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -2,22 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11820" yWindow="660" windowWidth="18420" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,11 +25,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -42,8 +40,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F4F4F"/>
-        <bgColor rgb="002F4F4F"/>
+        <fgColor rgb="FF2F4F4F"/>
+        <bgColor rgb="FF2F4F4F"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,23 +54,33 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -435,8 +443,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G77"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -477,6 +485,11 @@
           <t>Country</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +522,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -541,6 +559,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -573,6 +596,11 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -605,6 +633,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +670,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -669,6 +707,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -701,6 +744,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -733,6 +781,11 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -765,6 +818,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>7:1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -797,6 +855,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -829,6 +892,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -861,6 +929,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>5:1</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -893,6 +966,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -925,6 +1003,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -957,6 +1040,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -989,6 +1077,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1021,6 +1114,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1053,6 +1151,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1085,6 +1188,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1117,6 +1221,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1149,6 +1254,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1181,6 +1287,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1213,6 +1320,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1245,6 +1353,7 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1277,6 +1386,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1309,6 +1419,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1341,6 +1452,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1373,6 +1485,7 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1405,6 +1518,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1437,6 +1551,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1469,6 +1584,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1501,6 +1617,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1533,6 +1650,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1565,6 +1683,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1597,6 +1716,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1629,6 +1749,7 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1661,6 +1782,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1693,6 +1815,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1725,6 +1848,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1757,6 +1881,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1789,6 +1914,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1821,6 +1947,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1853,6 +1980,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1885,6 +2013,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1917,6 +2046,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1949,6 +2079,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1981,6 +2112,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2013,6 +2145,7 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2045,6 +2178,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2077,6 +2211,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2109,6 +2244,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2141,6 +2277,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2173,6 +2310,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2205,6 +2343,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2237,6 +2376,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2269,6 +2409,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2301,6 +2442,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2333,6 +2475,7 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2365,6 +2508,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2397,6 +2541,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2429,6 +2574,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2461,6 +2607,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2493,6 +2640,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2525,6 +2673,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2557,6 +2706,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2589,6 +2739,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2621,6 +2772,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2653,6 +2805,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2685,6 +2838,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2717,6 +2871,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2749,6 +2904,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2781,6 +2937,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2813,6 +2970,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2845,6 +3003,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2877,6 +3036,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2909,6 +3069,7 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G77" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
results: add final scores
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -1188,7 +1188,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>

<commit_message>
fix: partial team name matching for ESPN and football-data.org
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Canada vs Bosnia and Herzegovina</t>
+          <t>Canada vs Bosnia</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Switzerland vs Bosnia and Herzegovina</t>
+          <t>Switzerland vs Bosnia</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">

</xml_diff>

<commit_message>
feat: add MD3 games + backfill scores through Jun 22
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11820" yWindow="660" windowWidth="18420" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
@@ -26,6 +26,7 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
@@ -443,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -953,7 +954,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Spain vs Cabo Verde</t>
+          <t>Spain vs Cape Verde</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1225,7 +1226,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1258,7 +1263,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1291,7 +1300,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1324,7 +1337,11 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1357,7 +1374,11 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1390,7 +1411,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1423,7 +1448,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1456,7 +1485,11 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>6:0</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1489,7 +1522,11 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1522,7 +1559,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1555,7 +1596,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1588,7 +1633,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1621,7 +1670,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1654,7 +1707,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G34" s="2" t="n"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>5:1</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1687,7 +1744,11 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1720,7 +1781,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1753,7 +1818,11 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>0:4</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1786,7 +1855,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1819,7 +1892,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G39" s="2" t="n"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1839,7 +1916,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Uruguay vs Cabo Verde</t>
+          <t>Uruguay vs Cape Verde</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1852,7 +1929,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1885,7 +1966,11 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1918,7 +2003,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1951,7 +2040,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G43" s="2" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1984,7 +2077,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G44" s="2" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>3:2</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2017,7 +2114,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2154,60 +2255,59 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>June 28</t>
+          <t>June 24</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Switzerland vs Canada</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>BC Place Vancouver</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="n"/>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>June 28</t>
+          <t>June 24</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Bosnia vs Qatar</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>Seattle Stadium</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2215,32 +2315,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>June 29</t>
+          <t>June 24</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Morocco vs Haiti</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2248,32 +2347,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>June 29</t>
+          <t>June 24</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Scotland vs Brazil</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Philadelphia Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2281,98 +2379,95 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>June 30</t>
+          <t>June 24</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Czechia vs Mexico</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Houston Stadium</t>
+          <t>Estadio Banorte</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="n"/>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>June 30</t>
+          <t>June 24</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>South Africa vs South Korea</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>Estadio BBVA</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="n"/>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>July 1</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Ecuador vs Germany</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2380,32 +2475,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>July 1</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Curaçao vs Ivory Coast</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Seattle Stadium</t>
+          <t>Philadelphia Stadium</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2413,98 +2507,95 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>July 2</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Tunisia vs Netherlands</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Toronto Stadium</t>
+          <t>Kansas City Stadium</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="n"/>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>July 2</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Japan vs Sweden</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>BC Place Vancouver</t>
+          <t>Arlington Stadium</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="n"/>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>July 3</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Türkiye vs USA</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Kansas City Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2512,32 +2603,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>July 3</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Paraguay vs Australia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>Levi's Stadium</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2545,17 +2635,16 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>July 4</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2565,12 +2654,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Norway vs France</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Philadelphia Stadium</t>
+          <t>Massachusetts Stadium</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2578,98 +2667,95 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>July 4</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Senegal vs Iraq</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Houston Stadium</t>
+          <t>Toronto Stadium</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="n"/>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>July 5</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Uruguay vs Spain</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Estadio Akron</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="n"/>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>July 5</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Cape Verde vs Saudi Arabia</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>Houston Stadium</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2677,65 +2763,63 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>July 6</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>New Zealand vs Belgium</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>BC Place Vancouver</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="n"/>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>July 6</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Egypt vs Iran</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Seattle Stadium</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2743,32 +2827,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>July 7</t>
+          <t>June 27</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Panama vs England</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Seattle Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2776,32 +2859,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>July 7</t>
+          <t>June 27</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Croatia vs Ghana</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>Philadelphia Stadium</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -2809,32 +2891,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>July 9</t>
+          <t>June 27</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Colombia vs Portugal</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2842,32 +2923,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>July 10</t>
+          <t>June 27</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Congo DR vs Uzbekistan</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Los Angeles Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2875,32 +2955,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>July 11</t>
+          <t>June 27</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Jordan vs Argentina</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>Arlington Stadium</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2908,27 +2987,26 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>July 11</t>
+          <t>June 27</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Algeria vs Austria</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2941,22 +3019,21 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Semi-final</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>July 14</t>
+          <t>June 28</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2966,7 +3043,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -2979,17 +3056,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Semi-final</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>July 15</t>
+          <t>June 28</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2999,7 +3076,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Boston Stadium</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3012,17 +3089,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Third Place</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>July 18</t>
+          <t>June 29</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3032,7 +3109,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3045,35 +3122,827 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>June 29</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Philadelphia Stadium</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>June 30</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Houston Stadium</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>June 30</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>July 1</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>July 1</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Seattle Stadium</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>July 2</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Toronto Stadium</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>July 2</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>BC Place Vancouver</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>July 3</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Round of 32</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>July 3</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>July 4</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Philadelphia Stadium</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>July 4</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Houston Stadium</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>July 5</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>MetLife Stadium</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>July 5</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Boston Stadium</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>July 6</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>July 6</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>July 7</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Seattle Stadium</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Round of 16</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>July 7</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>July 9</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Boston Stadium</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>July 10</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>July 11</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>July 11</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>July 14</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>July 15</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Third Place</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>July 18</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
           <t>Final</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>July 19</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D101" t="inlineStr">
         <is>
           <t>TBD vs TBD</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>New York/New Jersey Stadium</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="n"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update Round of 32 confirmed matchups
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -3038,7 +3038,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>South Africa vs Canada</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Germany vs Paraguay</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>France vs Sweden</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Brazil vs Japan</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Ivory Coast vs Norway</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Argentina vs Cape Verde</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">

</xml_diff>

<commit_message>
backfill MD3 scores and insert missing Cabo Verde vs Saudi Arabia row
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2151,7 +2151,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G46" s="2" t="n"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>5:0</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2184,7 +2188,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G47" s="2" t="n"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2217,7 +2225,11 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="G48" s="2" t="n"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2250,7 +2262,11 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="G49" s="2" t="n"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2283,6 +2299,11 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2315,6 +2336,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2347,6 +2373,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>4:2</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2379,6 +2410,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2411,6 +2447,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2443,6 +2484,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2475,6 +2521,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2507,6 +2558,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2539,6 +2595,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2571,6 +2632,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2603,6 +2669,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>3:2</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2635,6 +2706,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2667,6 +2743,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2699,6 +2780,11 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>5:0</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2731,6 +2817,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2795,6 +2886,11 @@
           <t>Canada</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>1:5</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2827,6 +2923,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3023,35 +3124,29 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>June 28</t>
+          <t>June 26</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>South Africa vs Canada</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>SoFi Stadium</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="n"/>
+          <t>Cabo Verde vs Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3066,17 +3161,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Germany vs Paraguay</t>
+          <t>South Africa vs Canada</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3094,22 +3189,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>June 29</t>
+          <t>June 28</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>France vs Sweden</t>
+          <t>Germany vs Paraguay</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Boston Stadium</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3132,17 +3227,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>France vs Sweden</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Philadelphia Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3160,22 +3255,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>June 30</t>
+          <t>June 29</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Brazil vs Japan</t>
+          <t>TBD vs TBD</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Houston Stadium</t>
+          <t>Philadelphia Stadium</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3198,17 +3293,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Ivory Coast vs Norway</t>
+          <t>Brazil vs Japan</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>Houston Stadium</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3226,22 +3321,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>July 1</t>
+          <t>June 30</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Ivory Coast vs Norway</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Dallas Stadium</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3264,7 +3359,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3274,7 +3369,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Seattle Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3292,12 +3387,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>July 2</t>
+          <t>July 1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3307,12 +3402,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Toronto Stadium</t>
+          <t>Seattle Stadium</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="G82" s="2" t="n"/>
@@ -3330,7 +3425,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3340,7 +3435,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>BC Place Vancouver</t>
+          <t>Toronto Stadium</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3358,12 +3453,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>July 3</t>
+          <t>July 2</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3373,12 +3468,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Kansas City Stadium</t>
+          <t>BC Place Vancouver</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="G84" s="2" t="n"/>
@@ -3396,17 +3491,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Argentina vs Cape Verde</t>
+          <t>TBD vs TBD</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>Kansas City Stadium</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3419,27 +3514,27 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>July 4</t>
+          <t>July 3</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Argentina vs Cape Verde</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Philadelphia Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3462,7 +3557,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3472,7 +3567,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Houston Stadium</t>
+          <t>Philadelphia Stadium</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3490,12 +3585,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>July 5</t>
+          <t>July 4</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3505,7 +3600,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Houston Stadium</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3528,7 +3623,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3538,7 +3633,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3556,12 +3651,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>July 6</t>
+          <t>July 5</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3571,7 +3666,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>Boston Stadium</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3594,7 +3689,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3604,7 +3699,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Dallas Stadium</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3622,12 +3717,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>July 7</t>
+          <t>July 6</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3637,7 +3732,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Seattle Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3660,7 +3755,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3670,7 +3765,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>Seattle Stadium</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3683,17 +3778,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Round of 16</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>July 9</t>
+          <t>July 7</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3703,7 +3798,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -3721,7 +3816,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>July 10</t>
+          <t>July 9</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3736,7 +3831,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Los Angeles Stadium</t>
+          <t>Boston Stadium</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -3754,7 +3849,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>July 11</t>
+          <t>July 10</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3769,7 +3864,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>Los Angeles Stadium</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -3792,7 +3887,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3802,7 +3897,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Kansas City Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -3815,17 +3910,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Semi-final</t>
+          <t>Quarter-final</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>July 14</t>
+          <t>July 11</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3835,7 +3930,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>Kansas City Stadium</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -3853,7 +3948,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>July 15</t>
+          <t>July 14</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3868,7 +3963,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Dallas Stadium</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -3881,17 +3976,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Third Place</t>
+          <t>Semi-final</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>July 18</t>
+          <t>July 15</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3901,7 +3996,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3914,35 +4009,68 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
+          <t>Third Place</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>July 18</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>Final</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>July 19</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>TBD vs TBD</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>New York/New Jersey Stadium</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G101" s="2" t="n"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix knockout schedule: correct dates/times/venues from ESPN
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2960,6 +2960,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2992,6 +2997,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3151,35 +3161,29 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Round of 32</t>
+          <t>Group Stage</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>June 28</t>
+          <t>June 25</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>South Africa vs Canada</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>SoFi Stadium</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="n"/>
+          <t>Turkiye vs USA</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>3:2</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3194,17 +3198,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Germany vs Paraguay</t>
+          <t>South Africa vs Canada</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3212,7 +3216,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3232,12 +3235,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>France vs Sweden</t>
+          <t>Brazil vs Japan</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Houston Stadium</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3245,7 +3248,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3260,17 +3262,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Germany vs Paraguay</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Philadelphia Stadium</t>
+          <t>Boston Stadium</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3278,7 +3280,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3288,30 +3289,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>June 30</t>
+          <t>June 29</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Brazil vs Japan</t>
+          <t>Netherlands vs Morocco</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Houston Stadium</t>
+          <t>Monterrey Stadium</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="n"/>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3344,7 +3344,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3354,22 +3353,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>July 1</t>
+          <t>June 30</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>France vs Sweden</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3377,7 +3376,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3387,30 +3385,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>July 1</t>
+          <t>June 30</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Mexico vs Ecuador</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Seattle Stadium</t>
+          <t>Guadalajara Stadium</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="n"/>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3420,30 +3417,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>July 2</t>
+          <t>July 1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>England vs TBD</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Toronto Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="n"/>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3453,30 +3449,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>July 2</t>
+          <t>July 1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Belgium vs TBD</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>BC Place Vancouver</t>
+          <t>Seattle Stadium</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="n"/>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3486,22 +3481,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>July 3</t>
+          <t>July 1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>USA vs Bosnia-Herzegovina</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Kansas City Stadium</t>
+          <t>San Jose Stadium</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3509,7 +3504,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3519,22 +3513,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>July 3</t>
+          <t>July 2</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Argentina vs Cape Verde</t>
+          <t>Spain vs TBD</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3542,98 +3536,95 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>July 4</t>
+          <t>July 2</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>TBD vs Croatia</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Philadelphia Stadium</t>
+          <t>Toronto Stadium</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="n"/>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>July 4</t>
+          <t>July 2</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Switzerland vs TBD</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Houston Stadium</t>
+          <t>BC Place Vancouver</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="n"/>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>July 5</t>
+          <t>July 3</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Australia vs Egypt</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>MetLife Stadium</t>
+          <t>Dallas Stadium</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3641,32 +3632,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>July 5</t>
+          <t>July 3</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Argentina vs Cape Verde</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3674,32 +3664,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Round of 16</t>
+          <t>Round of 32</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>July 6</t>
+          <t>July 3</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>TBD vs Ghana</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>Kansas City Stadium</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3707,7 +3696,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3717,12 +3705,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>July 6</t>
+          <t>July 4</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3732,7 +3720,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Houston Stadium</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3740,7 +3728,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3750,12 +3737,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>July 7</t>
+          <t>July 4</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3765,7 +3752,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Seattle Stadium</t>
+          <t>Philadelphia Stadium</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3773,7 +3760,6 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3783,12 +3769,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>July 7</t>
+          <t>July 5</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3798,7 +3784,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>SoFi Stadium</t>
+          <t>MetLife Stadium</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -3806,22 +3792,21 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Round of 16</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>July 9</t>
+          <t>July 5</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3831,30 +3816,29 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Boston Stadium</t>
+          <t>Guadalajara Stadium</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G95" s="2" t="n"/>
+          <t>Mexico</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Round of 16</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>July 10</t>
+          <t>July 6</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3864,7 +3848,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Los Angeles Stadium</t>
+          <t>Dallas Stadium</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -3872,22 +3856,21 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Round of 16</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>July 11</t>
+          <t>July 6</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3897,7 +3880,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>Seattle Stadium</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -3905,22 +3888,21 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Quarter-final</t>
+          <t>Round of 16</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>July 11</t>
+          <t>July 7</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3930,7 +3912,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Kansas City Stadium</t>
+          <t>Atlanta Stadium</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -3938,22 +3920,21 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Semi-final</t>
+          <t>Round of 16</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>July 14</t>
+          <t>July 7</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3963,30 +3944,29 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Dallas Stadium</t>
+          <t>BC Place Vancouver</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G99" s="2" t="n"/>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Semi-final</t>
+          <t>Quarter-final</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>July 15</t>
+          <t>July 9</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3996,7 +3976,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Atlanta Stadium</t>
+          <t>Boston Stadium</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4004,22 +3984,21 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Third Place</t>
+          <t>Quarter-final</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>July 18</t>
+          <t>July 10</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4029,7 +4008,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>SoFi Stadium</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4037,40 +4016,198 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="G101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>July 11</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Quarter-final</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>July 11</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>July 14</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>July 15</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Third Place</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>July 18</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>TBD vs TBD</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
           <t>Final</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>July 19</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
         <is>
           <t>TBD vs TBD</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>New York/New Jersey Stadium</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G102" s="2" t="n"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>MetLife Stadium</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix group stage times; add timing gate test
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">

</xml_diff>

<commit_message>
sync xlsx and no-scores variant
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -3310,6 +3310,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>1:1, 3:4p</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3342,6 +3347,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>1:1, 2:3p</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3745,7 +3755,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Canada vs TBD</t>
+          <t>Canada vs Morocco</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -3777,7 +3787,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Paraguay vs TBD</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">

</xml_diff>

<commit_message>
update schedule + fix daemon trophy
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -3495,6 +3495,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3527,6 +3532,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>3:2</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3559,6 +3569,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3866,7 +3881,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Mexico vs TBD</t>
+          <t>Mexico vs England</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -3930,7 +3945,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>USA vs Belgium</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">

</xml_diff>

<commit_message>
fix Australia vs Egypt penalty score
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -3702,6 +3702,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>1:1, 2:4p</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">

</xml_diff>

<commit_message>
fix Mexico vs England kickoff time
</commit_message>
<xml_diff>
--- a/2026_FIFA_World_Cup_Schedule.xlsx
+++ b/2026_FIFA_World_Cup_Schedule.xlsx
@@ -3902,6 +3902,11 @@
           <t>USA</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3916,7 +3921,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4145,7 +4150,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>TBD vs TBD</t>
+          <t>Norway vs TBD</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">

</xml_diff>